<commit_message>
examine plots density impact
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/compare_models/smaller_network/demand_scenarios144.xlsx
+++ b/study_case_model/scenario_variables/compare_models/smaller_network/demand_scenarios144.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,27 +417,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
@@ -473,7 +461,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2298.02849180674</v>
+        <v>2350.925503922311</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +524,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1917.041419297289</v>
+        <v>2738.71744426434</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +587,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1194.306561430208</v>
+        <v>1246.570079200356</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +650,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2913.817913844815</v>
+        <v>1520.462985682129</v>
       </c>
     </row>
     <row r="12">
@@ -725,7 +713,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1859.507975165998</v>
+        <v>2247.23193822144</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +776,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>929.7589129152458</v>
+        <v>947.1530157355126</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +839,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2947.527689304435</v>
+        <v>1956.09681821819</v>
       </c>
     </row>
     <row r="21">
@@ -914,7 +902,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2460.460837491745</v>
+        <v>1660.600166340649</v>
       </c>
     </row>
     <row r="24">
@@ -977,7 +965,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>859.1576842195143</v>
+        <v>971.9604271629986</v>
       </c>
     </row>
     <row r="27">
@@ -1040,7 +1028,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2325.536026151579</v>
+        <v>2514.380649784153</v>
       </c>
     </row>
     <row r="30">
@@ -1103,7 +1091,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1721.949384312523</v>
+        <v>1482.66602827365</v>
       </c>
     </row>
     <row r="33">
@@ -1166,7 +1154,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>860.281073928923</v>
+        <v>1004.944329862179</v>
       </c>
     </row>
     <row r="36">

</xml_diff>